<commit_message>
Minor changes to CSV uploads and attachments
</commit_message>
<xml_diff>
--- a/backend/data/DSA1101_Sem1_2425_Final.xlsx
+++ b/backend/data/DSA1101_Sem1_2425_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhixin/Documents/y4s1/dsa3101/extracted_questions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhixin/Documents/y4s1/dsa3101/dsa3101-2510-quiz-02/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0458A9-A2D0-2A49-BEFC-4903E67E82BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2ADF11-B5AF-2643-A5AF-F1E11723AC38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{CA20E2D9-AC26-2B4B-A400-E03C0BFEE2BC}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{CA20E2D9-AC26-2B4B-A400-E03C0BFEE2BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Context" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="84">
   <si>
-    <t>Context ID</t>
-  </si>
-  <si>
     <t>Context Text</t>
   </si>
   <si>
@@ -324,6 +321,9 @@
   </si>
   <si>
     <t>Model Validation</t>
+  </si>
+  <si>
+    <t>Context ID</t>
   </si>
 </sst>
 </file>
@@ -359,12 +359,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,13 +707,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="136" x14ac:dyDescent="0.2">
@@ -722,10 +721,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="34" x14ac:dyDescent="0.2">
@@ -733,7 +732,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="272" x14ac:dyDescent="0.2">
@@ -741,10 +740,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="204" x14ac:dyDescent="0.2">
@@ -752,10 +751,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -768,9 +767,10 @@
   <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="29.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="29.5" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" customWidth="1"/>
     <col min="6" max="10" width="10.83203125" customWidth="1"/>
     <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
@@ -780,52 +780,52 @@
   <sheetData>
     <row r="1" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
+      <c r="D1" t="s">
+        <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
-        <v>12</v>
-      </c>
       <c r="P1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -838,20 +838,20 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>19</v>
+      <c r="D2" t="s">
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M2">
         <v>4</v>
       </c>
       <c r="N2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -864,20 +864,20 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>20</v>
+      <c r="D3" t="s">
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M3">
         <v>6</v>
       </c>
       <c r="N3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -890,35 +890,35 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>25</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>26</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>27</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>28</v>
-      </c>
-      <c r="J4" t="s">
-        <v>29</v>
       </c>
       <c r="M4">
         <v>2.5</v>
       </c>
       <c r="N4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
@@ -931,35 +931,35 @@
       <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>30</v>
+      <c r="D5" t="s">
+        <v>29</v>
       </c>
       <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
         <v>24</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>25</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>26</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>27</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>28</v>
-      </c>
-      <c r="J5" t="s">
-        <v>29</v>
       </c>
       <c r="M5">
         <v>2.5</v>
       </c>
       <c r="N5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
@@ -972,35 +972,35 @@
       <c r="C6">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>31</v>
+      <c r="D6" t="s">
+        <v>30</v>
       </c>
       <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>25</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>26</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>27</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>28</v>
-      </c>
-      <c r="J6" t="s">
-        <v>29</v>
       </c>
       <c r="M6">
         <v>2.5</v>
       </c>
       <c r="N6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
@@ -1013,35 +1013,35 @@
       <c r="C7">
         <v>4</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>32</v>
+      <c r="D7" t="s">
+        <v>31</v>
       </c>
       <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
         <v>24</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>25</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>26</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>27</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>28</v>
-      </c>
-      <c r="J7" t="s">
-        <v>29</v>
       </c>
       <c r="M7">
         <v>2.5</v>
       </c>
       <c r="N7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -1054,20 +1054,20 @@
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>35</v>
+      <c r="D8" t="s">
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M8">
         <v>2</v>
       </c>
       <c r="N8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -1080,20 +1080,20 @@
       <c r="C9">
         <v>2</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>36</v>
+      <c r="D9" t="s">
+        <v>35</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M9">
         <v>2</v>
       </c>
       <c r="N9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -1106,20 +1106,20 @@
       <c r="C10">
         <v>3</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>37</v>
+      <c r="D10" t="s">
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M10">
         <v>2</v>
       </c>
       <c r="N10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -1132,20 +1132,20 @@
       <c r="C11">
         <v>4</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>38</v>
+      <c r="D11" t="s">
+        <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M11">
         <v>4</v>
       </c>
       <c r="N11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -1158,20 +1158,20 @@
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>41</v>
+      <c r="D12" t="s">
+        <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M12">
         <v>2</v>
       </c>
       <c r="N12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -1184,20 +1184,20 @@
       <c r="C13">
         <v>2</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>43</v>
+      <c r="D13" t="s">
+        <v>42</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M13">
         <v>6</v>
       </c>
       <c r="N13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -1210,20 +1210,20 @@
       <c r="C14">
         <v>3</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>42</v>
+      <c r="D14" t="s">
+        <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M14">
         <v>4</v>
       </c>
       <c r="N14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -1236,20 +1236,20 @@
       <c r="C15">
         <v>4</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>44</v>
+      <c r="D15" t="s">
+        <v>43</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M15">
         <v>3</v>
       </c>
       <c r="N15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -1262,20 +1262,20 @@
       <c r="C16">
         <v>5</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>45</v>
+      <c r="D16" t="s">
+        <v>44</v>
       </c>
       <c r="E16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M16">
         <v>5</v>
       </c>
       <c r="N16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
@@ -1288,20 +1288,20 @@
       <c r="C17">
         <v>6</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>46</v>
+      <c r="D17" t="s">
+        <v>45</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M17">
         <v>2</v>
       </c>
       <c r="N17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
@@ -1314,20 +1314,20 @@
       <c r="C18">
         <v>7</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>47</v>
+      <c r="D18" t="s">
+        <v>46</v>
       </c>
       <c r="E18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M18">
         <v>4</v>
       </c>
       <c r="N18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
@@ -1340,20 +1340,20 @@
       <c r="C19">
         <v>8</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>48</v>
+      <c r="D19" t="s">
+        <v>47</v>
       </c>
       <c r="E19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M19">
         <v>4</v>
       </c>
       <c r="N19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
@@ -1366,20 +1366,20 @@
       <c r="C20">
         <v>9</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>53</v>
+      <c r="D20" t="s">
+        <v>52</v>
       </c>
       <c r="E20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M20">
         <v>3</v>
       </c>
       <c r="N20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
@@ -1392,20 +1392,20 @@
       <c r="C21">
         <v>10</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>49</v>
+      <c r="D21" t="s">
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M21">
         <v>3</v>
       </c>
       <c r="N21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
@@ -1418,20 +1418,20 @@
       <c r="C22">
         <v>11</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>50</v>
+      <c r="D22" t="s">
+        <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M22">
         <v>4</v>
       </c>
       <c r="N22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
@@ -1444,20 +1444,20 @@
       <c r="C23">
         <v>12</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>51</v>
+      <c r="D23" t="s">
+        <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M23">
         <v>5</v>
       </c>
       <c r="N23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
@@ -1470,20 +1470,20 @@
       <c r="C24">
         <v>13</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>52</v>
+      <c r="D24" t="s">
+        <v>51</v>
       </c>
       <c r="E24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M24">
         <v>5</v>
       </c>
       <c r="N24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
@@ -1496,20 +1496,20 @@
       <c r="C25">
         <v>14</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>54</v>
+      <c r="D25" t="s">
+        <v>53</v>
       </c>
       <c r="E25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M25">
         <v>3</v>
       </c>
       <c r="N25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
@@ -1522,20 +1522,20 @@
       <c r="C26">
         <v>15</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>55</v>
+      <c r="D26" t="s">
+        <v>54</v>
       </c>
       <c r="E26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M26">
         <v>4</v>
       </c>
       <c r="N26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
@@ -1548,20 +1548,20 @@
       <c r="C27">
         <v>16</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>56</v>
+      <c r="D27" t="s">
+        <v>55</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M27">
         <v>2</v>
       </c>
       <c r="N27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
@@ -1574,20 +1574,20 @@
       <c r="C28">
         <v>17</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>57</v>
+      <c r="D28" t="s">
+        <v>56</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M28">
         <v>3</v>
       </c>
       <c r="N28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
@@ -1600,20 +1600,20 @@
       <c r="C29">
         <v>18</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>58</v>
+      <c r="D29" t="s">
+        <v>57</v>
       </c>
       <c r="E29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M29">
         <v>3</v>
       </c>
       <c r="N29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
@@ -1626,20 +1626,20 @@
       <c r="C30">
         <v>19</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>60</v>
+      <c r="D30" t="s">
+        <v>59</v>
       </c>
       <c r="E30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M30">
         <v>3</v>
       </c>
       <c r="N30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="O30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
@@ -1652,20 +1652,20 @@
       <c r="C31">
         <v>20</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>59</v>
+      <c r="D31" t="s">
+        <v>58</v>
       </c>
       <c r="E31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M31">
         <v>2</v>
       </c>
       <c r="N31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>